<commit_message>
freelance: aggiorna la lista studi con i dati trovati (attività, contatti, bilanci) e aggiunge il foglio Fonti
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RNxVApXF9MzdDwSEC8TCy4
</commit_message>
<xml_diff>
--- a/freelance/studi-ingegneria.xlsx
+++ b/freelance/studi-ingegneria.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Studi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domande" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonti" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domande" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Studi'!$A$4:$N$44</definedName>
@@ -22,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +68,12 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -98,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -113,17 +120,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -493,16 +501,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="38" customWidth="1" min="9" max="9"/>
-    <col width="38" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="50" customWidth="1" min="14" max="14"/>
@@ -518,7 +526,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Obiettivo: parlare con colleghi della zona per capire quali aziende hanno problemi tecnici o documentali e se possono servire collaboratori esterni. Le colonne in blu vanno compilate a mano. 'Tipo' è una stima dal solo nome: va confermata. Una ricerca web non ha confermato l'esistenza degli studi tranne parzialmente per Barci Engineering. Il fatturato degli studi individuali non è pubblico.</t>
+          <t>Obiettivo: parlare con colleghi della zona per capire quali aziende hanno problemi tecnici o documentali e se servono collaboratori esterni. Le colonne in blu vanno compilate a mano. Dati raccolti da elenchi pubblici (28/10/2026): possono essere vecchi o discordanti, quindi vanno confermati con una telefonata. Priorità = affinità con il tuo profilo (elettrico/elettronico, industria), non qualità dello studio. Il fatturato degli studi individuali non è pubblico.</t>
         </is>
       </c>
     </row>
@@ -535,12 +543,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Tipo (stima dal nome)</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Indirizzo (come indicato)</t>
+          <t>Indirizzo</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -550,12 +558,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Telefono</t>
+          <t>Telefono (da elenchi)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Sito / contatto</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -570,12 +578,12 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Fonte / stato verifica</t>
+          <t>Priorità suggerita (1-3)</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Priorità suggerita (1-3)</t>
+          <t>Note di verifica</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -594,79 +602,83 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="78" customHeight="1">
+    <row r="5" ht="92" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Barci Engineering S.p.A.</t>
+          <t>Studio di ingegneria Monticone Ing. Marcello</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Società di ingegneria (S.p.A.)</t>
+          <t>Professionista singolo</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Via Tolstoj 86</t>
+          <t>Via Adda 18</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>San Giuliano Milanese</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>www.barciengineering.it</t>
+          <t>San Donato Milanese</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>02 36736620 (da elenchi; altri numeri discordanti)</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>monticone.eu</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Un elenco MePA (anno 2024) la dà con sede legale a Montalto Uffugo (CS), P.IVA 02444790782. Attività esatta e ruolo della sede di San Giuliano da verificare.</t>
+          <t>Progettazione e direzione lavori di impianti elettrici ed elettronici (rilevazione incendi, cablaggio strutturato), sicurezza sul lavoro e valutazione dei rischi.</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Non trovati. Per le S.p.A. il bilancio si può chiedere al Registro Imprese (Telemaco, copia bilancio 2,50 €).</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Elenco MePA (parziale); nessun dato su fatturato e dipendenti</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="n">
+          <t>Non pubblici (ditta individuale / professionista)</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="L5" s="7" t="n"/>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Il più vicino al tuo profilo (impianti elettrici/elettronici) e a casa tua. Verifica sul sito.</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="n"/>
+      <c r="M5" s="7" t="inlineStr">
         <is>
           <t>Da contattare</t>
         </is>
       </c>
-      <c r="N5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="78" customHeight="1">
+      <c r="N5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="92" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Studiora</t>
+          <t>Barci Engineering S.p.A.</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Studio (da verificare)</t>
+          <t>Società di ingegneria</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Via Emilia 24</t>
+          <t>Via Tolstoj 86</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -674,115 +686,127 @@
           <t>San Giuliano Milanese</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>barci.it</t>
+        </is>
+      </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Non verificato online</t>
+          <t>Progettazione di impianti elettrici e meccanici, condotte (pipeline), telecontrollo, infrastrutture civili, collaudi e perizie, protezioni elettriche, efficienza energetica. Qualifiche con Eni ed Enel Rete Gas.</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Non trovati</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>Ricerca web del 28/10/2026: nessun riscontro</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="6" t="inlineStr">
+          <t>Fatturato 2025 circa 18,1 M€, utile circa 2,9 M€ (ReportAziende); altra fonte: 14,4 M€ nel 2024. Dipendenti stimati 100–249 (altre fonti fino a 500). P.IVA 02444790782.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Sede legale a Montalto Uffugo (CS); un elenco la dà con sede a San Giuliano. Grande e strutturata: più difficile da avvicinare, ma strategica (settore energia). Contatto via LinkedIn o centralino.</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="n"/>
+      <c r="M6" s="7" t="inlineStr">
         <is>
           <t>Da contattare</t>
         </is>
       </c>
-      <c r="N6" s="6" t="n"/>
-    </row>
-    <row r="7" ht="78" customHeight="1">
+      <c r="N6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="92" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Ing. Lamanna Simone</t>
+          <t>DEAL Progetti S.r.l.</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Professionista singolo (probabile)</t>
+          <t>Società di ingegneria (microimpresa)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Via Molise 9</t>
+          <t>Via Mameli 2</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>San Giuliano Milanese</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
+          <t>Milano</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>02 783664 (da elenchi)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Non verificato online</t>
+          <t>Progettazione edile, di impianti e urbana; coordinamento della sicurezza e direzione lavori (ATECO 71.12.10). Pagine Bianche la associa all'Ing. Antonio De Marco.</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Non pubblici (professionista)</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>Ricerca non eseguita. Verifica sull'Albo dell'Ordine degli Ingegneri di Milano</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="n">
+          <t>Fatturato 2024 circa 213.302 € con utile di 4.078 €; 1 dipendente. Le fonti divergono (2021: 144.543 €). Costituita il 30/05/2019. P.IVA 10835040964.</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="6" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Società piccola; chiedi consigli all'ingegnere titolare.</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="n"/>
+      <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Da contattare</t>
         </is>
       </c>
-      <c r="N7" s="6" t="n"/>
-    </row>
-    <row r="8" ht="78" customHeight="1">
+      <c r="N7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="92" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Studio Ingegneria Lomanno</t>
+          <t>Studiora - Studio Ingegneria</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Studio (da verificare)</t>
+          <t>Studio di ingegneria</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Via Triulziana 38</t>
+          <t>Via Emilia 24</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>San Donato Milanese</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
+          <t>San Donato Milanese (negli elenchi; tu avevi indicato San Giuliano)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>393 0000868 (da elenco)</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Non verificato online</t>
+          <t>Non chiaro: gli elenchi lo classificano solo come studio di ingegneria. Compare anche nell'elenco di Opera.</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -790,39 +814,39 @@
           <t>Non trovati</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>Ricerca web del 28/10/2026: nessun riscontro</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="n">
+      <c r="J8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="6" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Verifica l'indirizzo e la specialità con una telefonata.</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="n"/>
+      <c r="M8" s="7" t="inlineStr">
         <is>
           <t>Da contattare</t>
         </is>
       </c>
-      <c r="N8" s="6" t="n"/>
-    </row>
-    <row r="9" ht="78" customHeight="1">
+      <c r="N8" s="7" t="n"/>
+    </row>
+    <row r="9" ht="92" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Monticone Ing. Marcello</t>
+          <t>Studio di ingegneria Lommano (indicato come 'Lomanno')</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Professionista singolo (probabile)</t>
+          <t>Ditta individuale</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Via Adda 18</t>
+          <t>Via Triulziana 38</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -830,51 +854,55 @@
           <t>San Donato Milanese</t>
         </is>
       </c>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>02 7000 2422 (da elenchi)</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Non verificato online</t>
+          <t>Ingegneria civile: prevenzione incendi, ingegneria della sicurezza antincendio, audit HSE. Titolare: Massimo Lommano, libero professionista (tecnico antincendio). Attivo dal 2000. Cerca personale per la prevenzione incendi (LinkedIn).</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Non pubblici (professionista)</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>Ricerca web del 28/10/2026: nessun riscontro</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="6" t="inlineStr">
+          <t>Non pubblici (ditta individuale / professionista)</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Specialità lontana da elettronica/RF, ma utile come conoscenza del territorio.</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="n"/>
+      <c r="M9" s="7" t="inlineStr">
         <is>
           <t>Da contattare</t>
         </is>
       </c>
-      <c r="N9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="78" customHeight="1">
+      <c r="N9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="92" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Studio Parodi</t>
+          <t>Studio Tecnico Parodi (Ing. Furio Parodi)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Studio (da verificare)</t>
+          <t>Professionista singolo</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Via Libertà (n. civico da trovare)</t>
+          <t>Via/Viale della Libertà 68 (le fonti divergono sul nome della via)</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -882,87 +910,99 @@
           <t>San Donato Milanese</t>
         </is>
       </c>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>339 6439555 (da elenchi)</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>studio-parodi.it</t>
+        </is>
+      </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Non verificato online</t>
+          <t>Progettazione e direzione lavori per ristrutturazioni (CILA, SCIA, permessi), pratiche per i bonus fiscali, prevenzione incendi, catasto, certificazioni energetiche, perizie. Attivo dal 2010.</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Non trovati</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>Ricerca web del 28/10/2026: nessun riscontro. Numero civico non trovato: guardare su Google Maps o sulla scheda Pagine Gialle</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="6" t="inlineStr">
+          <t>Non pubblici (ditta individuale / professionista)</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Specialità edilizia residenziale: meno rilevante per te.</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="n"/>
+      <c r="M10" s="7" t="inlineStr">
         <is>
           <t>Da contattare</t>
         </is>
       </c>
-      <c r="N10" s="6" t="n"/>
-    </row>
-    <row r="11" ht="78" customHeight="1">
+      <c r="N10" s="7" t="n"/>
+    </row>
+    <row r="11" ht="92" customHeight="1">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>DEAL Progetti</t>
+          <t>Studio Lamanna Simone</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Società (da verificare)</t>
+          <t>Probabile geometra (le fonti discordano: 'Ing.' o 'Geometra')</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Via Mameli 2</t>
+          <t>Via Molise 9 (coworking), Sesto Ulteriano</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Milano</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
+          <t>San Giuliano Milanese</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>geomlamannasimone.it</t>
+        </is>
+      </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Non verificato online</t>
+          <t>Libero professionista: pratiche comunali, certificazioni energetiche, pratiche catastali. Sede legale in un coworking di Via Molise 9.</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Non trovati</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>Ricerca web del 28/10/2026: nessun riscontro</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="n">
+          <t>Non pubblici (ditta individuale / professionista)</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="6" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Il sito è intestato a 'Geometra Lamanna Simone': verifica il titolo sull'albo prima di contattarlo come ingegnere.</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="n"/>
+      <c r="M11" s="7" t="inlineStr">
         <is>
           <t>Da contattare</t>
         </is>
       </c>
-      <c r="N11" s="6" t="n"/>
-    </row>
-    <row r="12" ht="78" customHeight="1">
+      <c r="N11" s="7" t="n"/>
+    </row>
+    <row r="12" ht="92" customHeight="1">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
@@ -973,7 +1013,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Professionista singolo (probabile)</t>
+          <t>Da verificare</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -986,545 +1026,545 @@
           <t>Milano</t>
         </is>
       </c>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Non verificato online</t>
+          <t>Non trovato: nessun riscontro per questo nome. 'Carlo Rota' (CRC Engineering, zona Como) e Studio Rota Srl (Bergamo) sono persone/società diverse.</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Non pubblici (professionista)</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>Ricerca web del 28/10/2026: nessun riscontro</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="n">
+          <t>Non trovati</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="6" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Controlla sull'Albo dell'Ordine degli Ingegneri di Milano o su Pagine Gialle.</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="n"/>
+      <c r="M12" s="7" t="inlineStr">
         <is>
           <t>Da contattare</t>
         </is>
       </c>
-      <c r="N12" s="6" t="n"/>
+      <c r="N12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="6" t="n"/>
-      <c r="J13" s="6" t="n"/>
-      <c r="K13" s="6" t="n"/>
-      <c r="L13" s="6" t="n"/>
-      <c r="M13" s="6" t="n"/>
-      <c r="N13" s="6" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" s="7" t="n"/>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="6" t="n"/>
-      <c r="J14" s="6" t="n"/>
-      <c r="K14" s="6" t="n"/>
-      <c r="L14" s="6" t="n"/>
-      <c r="M14" s="6" t="n"/>
-      <c r="N14" s="6" t="n"/>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="7" t="n"/>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="6" t="n"/>
-      <c r="J15" s="6" t="n"/>
-      <c r="K15" s="6" t="n"/>
-      <c r="L15" s="6" t="n"/>
-      <c r="M15" s="6" t="n"/>
-      <c r="N15" s="6" t="n"/>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
+      <c r="J15" s="7" t="n"/>
+      <c r="K15" s="7" t="n"/>
+      <c r="L15" s="7" t="n"/>
+      <c r="M15" s="7" t="n"/>
+      <c r="N15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="6" t="n"/>
-      <c r="J16" s="6" t="n"/>
-      <c r="K16" s="6" t="n"/>
-      <c r="L16" s="6" t="n"/>
-      <c r="M16" s="6" t="n"/>
-      <c r="N16" s="6" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+      <c r="J16" s="7" t="n"/>
+      <c r="K16" s="7" t="n"/>
+      <c r="L16" s="7" t="n"/>
+      <c r="M16" s="7" t="n"/>
+      <c r="N16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="n"/>
-      <c r="J17" s="6" t="n"/>
-      <c r="K17" s="6" t="n"/>
-      <c r="L17" s="6" t="n"/>
-      <c r="M17" s="6" t="n"/>
-      <c r="N17" s="6" t="n"/>
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="7" t="n"/>
+      <c r="J17" s="7" t="n"/>
+      <c r="K17" s="7" t="n"/>
+      <c r="L17" s="7" t="n"/>
+      <c r="M17" s="7" t="n"/>
+      <c r="N17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="6" t="n"/>
-      <c r="J18" s="6" t="n"/>
-      <c r="K18" s="6" t="n"/>
-      <c r="L18" s="6" t="n"/>
-      <c r="M18" s="6" t="n"/>
-      <c r="N18" s="6" t="n"/>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="7" t="n"/>
+      <c r="K18" s="7" t="n"/>
+      <c r="L18" s="7" t="n"/>
+      <c r="M18" s="7" t="n"/>
+      <c r="N18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="6" t="n"/>
-      <c r="H19" s="6" t="n"/>
-      <c r="I19" s="6" t="n"/>
-      <c r="J19" s="6" t="n"/>
-      <c r="K19" s="6" t="n"/>
-      <c r="L19" s="6" t="n"/>
-      <c r="M19" s="6" t="n"/>
-      <c r="N19" s="6" t="n"/>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
+      <c r="J19" s="7" t="n"/>
+      <c r="K19" s="7" t="n"/>
+      <c r="L19" s="7" t="n"/>
+      <c r="M19" s="7" t="n"/>
+      <c r="N19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n"/>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="6" t="n"/>
-      <c r="J20" s="6" t="n"/>
-      <c r="K20" s="6" t="n"/>
-      <c r="L20" s="6" t="n"/>
-      <c r="M20" s="6" t="n"/>
-      <c r="N20" s="6" t="n"/>
+      <c r="B20" s="7" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="n"/>
+      <c r="I20" s="7" t="n"/>
+      <c r="J20" s="7" t="n"/>
+      <c r="K20" s="7" t="n"/>
+      <c r="L20" s="7" t="n"/>
+      <c r="M20" s="7" t="n"/>
+      <c r="N20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="6" t="n"/>
-      <c r="I21" s="6" t="n"/>
-      <c r="J21" s="6" t="n"/>
-      <c r="K21" s="6" t="n"/>
-      <c r="L21" s="6" t="n"/>
-      <c r="M21" s="6" t="n"/>
-      <c r="N21" s="6" t="n"/>
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="7" t="n"/>
+      <c r="J21" s="7" t="n"/>
+      <c r="K21" s="7" t="n"/>
+      <c r="L21" s="7" t="n"/>
+      <c r="M21" s="7" t="n"/>
+      <c r="N21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n"/>
-      <c r="B22" s="6" t="n"/>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="n"/>
-      <c r="H22" s="6" t="n"/>
-      <c r="I22" s="6" t="n"/>
-      <c r="J22" s="6" t="n"/>
-      <c r="K22" s="6" t="n"/>
-      <c r="L22" s="6" t="n"/>
-      <c r="M22" s="6" t="n"/>
-      <c r="N22" s="6" t="n"/>
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="7" t="n"/>
+      <c r="J22" s="7" t="n"/>
+      <c r="K22" s="7" t="n"/>
+      <c r="L22" s="7" t="n"/>
+      <c r="M22" s="7" t="n"/>
+      <c r="N22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" s="6" t="n"/>
-      <c r="I23" s="6" t="n"/>
-      <c r="J23" s="6" t="n"/>
-      <c r="K23" s="6" t="n"/>
-      <c r="L23" s="6" t="n"/>
-      <c r="M23" s="6" t="n"/>
-      <c r="N23" s="6" t="n"/>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="7" t="n"/>
+      <c r="J23" s="7" t="n"/>
+      <c r="K23" s="7" t="n"/>
+      <c r="L23" s="7" t="n"/>
+      <c r="M23" s="7" t="n"/>
+      <c r="N23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n"/>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6" t="n"/>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="n"/>
-      <c r="G24" s="6" t="n"/>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="6" t="n"/>
-      <c r="J24" s="6" t="n"/>
-      <c r="K24" s="6" t="n"/>
-      <c r="L24" s="6" t="n"/>
-      <c r="M24" s="6" t="n"/>
-      <c r="N24" s="6" t="n"/>
+      <c r="B24" s="7" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="7" t="n"/>
+      <c r="I24" s="7" t="n"/>
+      <c r="J24" s="7" t="n"/>
+      <c r="K24" s="7" t="n"/>
+      <c r="L24" s="7" t="n"/>
+      <c r="M24" s="7" t="n"/>
+      <c r="N24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n"/>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
-      <c r="I25" s="6" t="n"/>
-      <c r="J25" s="6" t="n"/>
-      <c r="K25" s="6" t="n"/>
-      <c r="L25" s="6" t="n"/>
-      <c r="M25" s="6" t="n"/>
-      <c r="N25" s="6" t="n"/>
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="7" t="n"/>
+      <c r="J25" s="7" t="n"/>
+      <c r="K25" s="7" t="n"/>
+      <c r="L25" s="7" t="n"/>
+      <c r="M25" s="7" t="n"/>
+      <c r="N25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n"/>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
-      <c r="I26" s="6" t="n"/>
-      <c r="J26" s="6" t="n"/>
-      <c r="K26" s="6" t="n"/>
-      <c r="L26" s="6" t="n"/>
-      <c r="M26" s="6" t="n"/>
-      <c r="N26" s="6" t="n"/>
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="7" t="n"/>
+      <c r="J26" s="7" t="n"/>
+      <c r="K26" s="7" t="n"/>
+      <c r="L26" s="7" t="n"/>
+      <c r="M26" s="7" t="n"/>
+      <c r="N26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n"/>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="6" t="n"/>
-      <c r="I27" s="6" t="n"/>
-      <c r="J27" s="6" t="n"/>
-      <c r="K27" s="6" t="n"/>
-      <c r="L27" s="6" t="n"/>
-      <c r="M27" s="6" t="n"/>
-      <c r="N27" s="6" t="n"/>
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="n"/>
+      <c r="H27" s="7" t="n"/>
+      <c r="I27" s="7" t="n"/>
+      <c r="J27" s="7" t="n"/>
+      <c r="K27" s="7" t="n"/>
+      <c r="L27" s="7" t="n"/>
+      <c r="M27" s="7" t="n"/>
+      <c r="N27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n"/>
-      <c r="B28" s="6" t="n"/>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="6" t="n"/>
-      <c r="I28" s="6" t="n"/>
-      <c r="J28" s="6" t="n"/>
-      <c r="K28" s="6" t="n"/>
-      <c r="L28" s="6" t="n"/>
-      <c r="M28" s="6" t="n"/>
-      <c r="N28" s="6" t="n"/>
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="n"/>
+      <c r="H28" s="7" t="n"/>
+      <c r="I28" s="7" t="n"/>
+      <c r="J28" s="7" t="n"/>
+      <c r="K28" s="7" t="n"/>
+      <c r="L28" s="7" t="n"/>
+      <c r="M28" s="7" t="n"/>
+      <c r="N28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n"/>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="6" t="n"/>
-      <c r="I29" s="6" t="n"/>
-      <c r="J29" s="6" t="n"/>
-      <c r="K29" s="6" t="n"/>
-      <c r="L29" s="6" t="n"/>
-      <c r="M29" s="6" t="n"/>
-      <c r="N29" s="6" t="n"/>
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="n"/>
+      <c r="H29" s="7" t="n"/>
+      <c r="I29" s="7" t="n"/>
+      <c r="J29" s="7" t="n"/>
+      <c r="K29" s="7" t="n"/>
+      <c r="L29" s="7" t="n"/>
+      <c r="M29" s="7" t="n"/>
+      <c r="N29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n"/>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="6" t="n"/>
-      <c r="J30" s="6" t="n"/>
-      <c r="K30" s="6" t="n"/>
-      <c r="L30" s="6" t="n"/>
-      <c r="M30" s="6" t="n"/>
-      <c r="N30" s="6" t="n"/>
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="7" t="n"/>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="7" t="n"/>
+      <c r="H30" s="7" t="n"/>
+      <c r="I30" s="7" t="n"/>
+      <c r="J30" s="7" t="n"/>
+      <c r="K30" s="7" t="n"/>
+      <c r="L30" s="7" t="n"/>
+      <c r="M30" s="7" t="n"/>
+      <c r="N30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n"/>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="6" t="n"/>
-      <c r="H31" s="6" t="n"/>
-      <c r="I31" s="6" t="n"/>
-      <c r="J31" s="6" t="n"/>
-      <c r="K31" s="6" t="n"/>
-      <c r="L31" s="6" t="n"/>
-      <c r="M31" s="6" t="n"/>
-      <c r="N31" s="6" t="n"/>
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="n"/>
+      <c r="H31" s="7" t="n"/>
+      <c r="I31" s="7" t="n"/>
+      <c r="J31" s="7" t="n"/>
+      <c r="K31" s="7" t="n"/>
+      <c r="L31" s="7" t="n"/>
+      <c r="M31" s="7" t="n"/>
+      <c r="N31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n"/>
-      <c r="B32" s="6" t="n"/>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
-      <c r="H32" s="6" t="n"/>
-      <c r="I32" s="6" t="n"/>
-      <c r="J32" s="6" t="n"/>
-      <c r="K32" s="6" t="n"/>
-      <c r="L32" s="6" t="n"/>
-      <c r="M32" s="6" t="n"/>
-      <c r="N32" s="6" t="n"/>
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="7" t="n"/>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="7" t="n"/>
+      <c r="H32" s="7" t="n"/>
+      <c r="I32" s="7" t="n"/>
+      <c r="J32" s="7" t="n"/>
+      <c r="K32" s="7" t="n"/>
+      <c r="L32" s="7" t="n"/>
+      <c r="M32" s="7" t="n"/>
+      <c r="N32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n"/>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6" t="n"/>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="6" t="n"/>
-      <c r="H33" s="6" t="n"/>
-      <c r="I33" s="6" t="n"/>
-      <c r="J33" s="6" t="n"/>
-      <c r="K33" s="6" t="n"/>
-      <c r="L33" s="6" t="n"/>
-      <c r="M33" s="6" t="n"/>
-      <c r="N33" s="6" t="n"/>
+      <c r="B33" s="7" t="n"/>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="7" t="n"/>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="7" t="n"/>
+      <c r="H33" s="7" t="n"/>
+      <c r="I33" s="7" t="n"/>
+      <c r="J33" s="7" t="n"/>
+      <c r="K33" s="7" t="n"/>
+      <c r="L33" s="7" t="n"/>
+      <c r="M33" s="7" t="n"/>
+      <c r="N33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n"/>
-      <c r="B34" s="6" t="n"/>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="6" t="n"/>
-      <c r="H34" s="6" t="n"/>
-      <c r="I34" s="6" t="n"/>
-      <c r="J34" s="6" t="n"/>
-      <c r="K34" s="6" t="n"/>
-      <c r="L34" s="6" t="n"/>
-      <c r="M34" s="6" t="n"/>
-      <c r="N34" s="6" t="n"/>
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="7" t="n"/>
+      <c r="H34" s="7" t="n"/>
+      <c r="I34" s="7" t="n"/>
+      <c r="J34" s="7" t="n"/>
+      <c r="K34" s="7" t="n"/>
+      <c r="L34" s="7" t="n"/>
+      <c r="M34" s="7" t="n"/>
+      <c r="N34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n"/>
-      <c r="B35" s="6" t="n"/>
-      <c r="C35" s="6" t="n"/>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="6" t="n"/>
-      <c r="G35" s="6" t="n"/>
-      <c r="H35" s="6" t="n"/>
-      <c r="I35" s="6" t="n"/>
-      <c r="J35" s="6" t="n"/>
-      <c r="K35" s="6" t="n"/>
-      <c r="L35" s="6" t="n"/>
-      <c r="M35" s="6" t="n"/>
-      <c r="N35" s="6" t="n"/>
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="n"/>
+      <c r="G35" s="7" t="n"/>
+      <c r="H35" s="7" t="n"/>
+      <c r="I35" s="7" t="n"/>
+      <c r="J35" s="7" t="n"/>
+      <c r="K35" s="7" t="n"/>
+      <c r="L35" s="7" t="n"/>
+      <c r="M35" s="7" t="n"/>
+      <c r="N35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n"/>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="6" t="n"/>
-      <c r="D36" s="6" t="n"/>
-      <c r="E36" s="6" t="n"/>
-      <c r="F36" s="6" t="n"/>
-      <c r="G36" s="6" t="n"/>
-      <c r="H36" s="6" t="n"/>
-      <c r="I36" s="6" t="n"/>
-      <c r="J36" s="6" t="n"/>
-      <c r="K36" s="6" t="n"/>
-      <c r="L36" s="6" t="n"/>
-      <c r="M36" s="6" t="n"/>
-      <c r="N36" s="6" t="n"/>
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="7" t="n"/>
+      <c r="E36" s="7" t="n"/>
+      <c r="F36" s="7" t="n"/>
+      <c r="G36" s="7" t="n"/>
+      <c r="H36" s="7" t="n"/>
+      <c r="I36" s="7" t="n"/>
+      <c r="J36" s="7" t="n"/>
+      <c r="K36" s="7" t="n"/>
+      <c r="L36" s="7" t="n"/>
+      <c r="M36" s="7" t="n"/>
+      <c r="N36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n"/>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="6" t="n"/>
-      <c r="D37" s="6" t="n"/>
-      <c r="E37" s="6" t="n"/>
-      <c r="F37" s="6" t="n"/>
-      <c r="G37" s="6" t="n"/>
-      <c r="H37" s="6" t="n"/>
-      <c r="I37" s="6" t="n"/>
-      <c r="J37" s="6" t="n"/>
-      <c r="K37" s="6" t="n"/>
-      <c r="L37" s="6" t="n"/>
-      <c r="M37" s="6" t="n"/>
-      <c r="N37" s="6" t="n"/>
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="7" t="n"/>
+      <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="n"/>
+      <c r="G37" s="7" t="n"/>
+      <c r="H37" s="7" t="n"/>
+      <c r="I37" s="7" t="n"/>
+      <c r="J37" s="7" t="n"/>
+      <c r="K37" s="7" t="n"/>
+      <c r="L37" s="7" t="n"/>
+      <c r="M37" s="7" t="n"/>
+      <c r="N37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n"/>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="6" t="n"/>
-      <c r="E38" s="6" t="n"/>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="6" t="n"/>
-      <c r="H38" s="6" t="n"/>
-      <c r="I38" s="6" t="n"/>
-      <c r="J38" s="6" t="n"/>
-      <c r="K38" s="6" t="n"/>
-      <c r="L38" s="6" t="n"/>
-      <c r="M38" s="6" t="n"/>
-      <c r="N38" s="6" t="n"/>
+      <c r="B38" s="7" t="n"/>
+      <c r="C38" s="7" t="n"/>
+      <c r="D38" s="7" t="n"/>
+      <c r="E38" s="7" t="n"/>
+      <c r="F38" s="7" t="n"/>
+      <c r="G38" s="7" t="n"/>
+      <c r="H38" s="7" t="n"/>
+      <c r="I38" s="7" t="n"/>
+      <c r="J38" s="7" t="n"/>
+      <c r="K38" s="7" t="n"/>
+      <c r="L38" s="7" t="n"/>
+      <c r="M38" s="7" t="n"/>
+      <c r="N38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n"/>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="6" t="n"/>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="6" t="n"/>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" s="6" t="n"/>
-      <c r="H39" s="6" t="n"/>
-      <c r="I39" s="6" t="n"/>
-      <c r="J39" s="6" t="n"/>
-      <c r="K39" s="6" t="n"/>
-      <c r="L39" s="6" t="n"/>
-      <c r="M39" s="6" t="n"/>
-      <c r="N39" s="6" t="n"/>
+      <c r="B39" s="7" t="n"/>
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="7" t="n"/>
+      <c r="E39" s="7" t="n"/>
+      <c r="F39" s="7" t="n"/>
+      <c r="G39" s="7" t="n"/>
+      <c r="H39" s="7" t="n"/>
+      <c r="I39" s="7" t="n"/>
+      <c r="J39" s="7" t="n"/>
+      <c r="K39" s="7" t="n"/>
+      <c r="L39" s="7" t="n"/>
+      <c r="M39" s="7" t="n"/>
+      <c r="N39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n"/>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="6" t="n"/>
-      <c r="D40" s="6" t="n"/>
-      <c r="E40" s="6" t="n"/>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="6" t="n"/>
-      <c r="H40" s="6" t="n"/>
-      <c r="I40" s="6" t="n"/>
-      <c r="J40" s="6" t="n"/>
-      <c r="K40" s="6" t="n"/>
-      <c r="L40" s="6" t="n"/>
-      <c r="M40" s="6" t="n"/>
-      <c r="N40" s="6" t="n"/>
+      <c r="B40" s="7" t="n"/>
+      <c r="C40" s="7" t="n"/>
+      <c r="D40" s="7" t="n"/>
+      <c r="E40" s="7" t="n"/>
+      <c r="F40" s="7" t="n"/>
+      <c r="G40" s="7" t="n"/>
+      <c r="H40" s="7" t="n"/>
+      <c r="I40" s="7" t="n"/>
+      <c r="J40" s="7" t="n"/>
+      <c r="K40" s="7" t="n"/>
+      <c r="L40" s="7" t="n"/>
+      <c r="M40" s="7" t="n"/>
+      <c r="N40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n"/>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="6" t="n"/>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="6" t="n"/>
-      <c r="F41" s="6" t="n"/>
-      <c r="G41" s="6" t="n"/>
-      <c r="H41" s="6" t="n"/>
-      <c r="I41" s="6" t="n"/>
-      <c r="J41" s="6" t="n"/>
-      <c r="K41" s="6" t="n"/>
-      <c r="L41" s="6" t="n"/>
-      <c r="M41" s="6" t="n"/>
-      <c r="N41" s="6" t="n"/>
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="7" t="n"/>
+      <c r="D41" s="7" t="n"/>
+      <c r="E41" s="7" t="n"/>
+      <c r="F41" s="7" t="n"/>
+      <c r="G41" s="7" t="n"/>
+      <c r="H41" s="7" t="n"/>
+      <c r="I41" s="7" t="n"/>
+      <c r="J41" s="7" t="n"/>
+      <c r="K41" s="7" t="n"/>
+      <c r="L41" s="7" t="n"/>
+      <c r="M41" s="7" t="n"/>
+      <c r="N41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n"/>
-      <c r="B42" s="6" t="n"/>
-      <c r="C42" s="6" t="n"/>
-      <c r="D42" s="6" t="n"/>
-      <c r="E42" s="6" t="n"/>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="6" t="n"/>
-      <c r="H42" s="6" t="n"/>
-      <c r="I42" s="6" t="n"/>
-      <c r="J42" s="6" t="n"/>
-      <c r="K42" s="6" t="n"/>
-      <c r="L42" s="6" t="n"/>
-      <c r="M42" s="6" t="n"/>
-      <c r="N42" s="6" t="n"/>
+      <c r="B42" s="7" t="n"/>
+      <c r="C42" s="7" t="n"/>
+      <c r="D42" s="7" t="n"/>
+      <c r="E42" s="7" t="n"/>
+      <c r="F42" s="7" t="n"/>
+      <c r="G42" s="7" t="n"/>
+      <c r="H42" s="7" t="n"/>
+      <c r="I42" s="7" t="n"/>
+      <c r="J42" s="7" t="n"/>
+      <c r="K42" s="7" t="n"/>
+      <c r="L42" s="7" t="n"/>
+      <c r="M42" s="7" t="n"/>
+      <c r="N42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n"/>
-      <c r="B43" s="6" t="n"/>
-      <c r="C43" s="6" t="n"/>
-      <c r="D43" s="6" t="n"/>
-      <c r="E43" s="6" t="n"/>
-      <c r="F43" s="6" t="n"/>
-      <c r="G43" s="6" t="n"/>
-      <c r="H43" s="6" t="n"/>
-      <c r="I43" s="6" t="n"/>
-      <c r="J43" s="6" t="n"/>
-      <c r="K43" s="6" t="n"/>
-      <c r="L43" s="6" t="n"/>
-      <c r="M43" s="6" t="n"/>
-      <c r="N43" s="6" t="n"/>
+      <c r="B43" s="7" t="n"/>
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="7" t="n"/>
+      <c r="E43" s="7" t="n"/>
+      <c r="F43" s="7" t="n"/>
+      <c r="G43" s="7" t="n"/>
+      <c r="H43" s="7" t="n"/>
+      <c r="I43" s="7" t="n"/>
+      <c r="J43" s="7" t="n"/>
+      <c r="K43" s="7" t="n"/>
+      <c r="L43" s="7" t="n"/>
+      <c r="M43" s="7" t="n"/>
+      <c r="N43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n"/>
-      <c r="B44" s="6" t="n"/>
-      <c r="C44" s="6" t="n"/>
-      <c r="D44" s="6" t="n"/>
-      <c r="E44" s="6" t="n"/>
-      <c r="F44" s="6" t="n"/>
-      <c r="G44" s="6" t="n"/>
-      <c r="H44" s="6" t="n"/>
-      <c r="I44" s="6" t="n"/>
-      <c r="J44" s="6" t="n"/>
-      <c r="K44" s="6" t="n"/>
-      <c r="L44" s="6" t="n"/>
-      <c r="M44" s="6" t="n"/>
-      <c r="N44" s="6" t="n"/>
+      <c r="B44" s="7" t="n"/>
+      <c r="C44" s="7" t="n"/>
+      <c r="D44" s="7" t="n"/>
+      <c r="E44" s="7" t="n"/>
+      <c r="F44" s="7" t="n"/>
+      <c r="G44" s="7" t="n"/>
+      <c r="H44" s="7" t="n"/>
+      <c r="I44" s="7" t="n"/>
+      <c r="J44" s="7" t="n"/>
+      <c r="K44" s="7" t="n"/>
+      <c r="L44" s="7" t="n"/>
+      <c r="M44" s="7" t="n"/>
+      <c r="N44" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:N44"/>
@@ -1547,6 +1587,224 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Fonti consultate (28/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Studio di ingegneria Monticone Ing. Marcello</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>https://aziende.virgilio.it/ingegneria/san-donato-milanese-mi/studio-ingegneria-monticone-ing-marcello</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>https://www.misterimprese.it/lombardia/milano/san-donato-milanese/ingegneri-studi/2576926.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Barci Engineering S.p.A.</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>https://barci.it/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>https://barci.it/qualifiche/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>https://www.reportaziende.it/barci_engineering_spa_cs_02444790782</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.aziende.it/barci-engineering-societa-a-responsabilita</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>DEAL Progetti S.r.l.</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>https://atoka.io/public/it/azienda/deal-progetti-srl/0eb9c851cbc5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>https://www.fatturatoitalia.it/deal-progetti-srl-10835040964</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>https://www.paginebianche.it/scheda/milano/de-marco-ing-antonio-deal-progetti.362945</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Studiora - Studio Ingegneria</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>https://www.reteimprese.it/ingegneri/san-donato-milanese</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>https://www.reteimprese.it/ingegneri/opera</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Studio di ingegneria Lommano</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>https://trova-aperto.it/san-donato-milanese/studio-di-ingegneria-lommano-2187902</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>https://it.linkedin.com/company/studio-di-ingegneria-lommano</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>https://firmania.it/san-donato-milanese/studio-di-ingegneria-lommano-4110959</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Studio Tecnico Parodi</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>https://www.studio-parodi.it/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>https://www.studio-parodi.it/certificazione-energetica-ape-milano/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Studio Lamanna Simone</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>http://www.geomlamannasimone.it/contatti</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/inglamanna/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Andrea Carlo Rota</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Nessuna fonte pertinente trovata</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId18"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1569,7 +1827,7 @@
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>«Buongiorno, sono un ingegnere delle telecomunicazioni della zona e sto avviando un'attività mia di automazione e analisi dati. Vorrei farle tre domande da collega, 15 minuti, quando le è comodo.»</t>
         </is>
@@ -1586,7 +1844,7 @@
       <c r="A7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Che tipo di clienti (PMI, industrie) avete in zona?</t>
         </is>
@@ -1596,7 +1854,7 @@
       <c r="A8" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Quali attività ripetitive o documenti vi fanno perdere più tempo?</t>
         </is>
@@ -1606,7 +1864,7 @@
       <c r="A9" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Vi capita di avere bisogno di collaboratori esterni per calcoli, CAD o automazioni?</t>
         </is>
@@ -1616,7 +1874,7 @@
       <c r="A10" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Come avete cominciato? Cosa vi sarebbe servito sapere all'inizio?</t>
         </is>
@@ -1626,7 +1884,7 @@
       <c r="A11" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Conoscete aziende della zona con problemi tecnici o di gestione che potrei ascoltare?</t>
         </is>
@@ -1643,7 +1901,7 @@
       <c r="A14" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Professionisti: Albo dell'Ordine degli Ingegneri della Provincia di Milano (ricerca pubblica per nome).</t>
         </is>
@@ -1653,7 +1911,7 @@
       <c r="A15" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Società: Registro Imprese, 'Trova impresa' su registroimprese.it (attività, ATECO, stato).</t>
         </is>
@@ -1663,7 +1921,7 @@
       <c r="A16" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Bilancio di una S.r.l./S.p.A.: Telemaco, copia del bilancio 2,50 €; visura ordinaria società di capitali 5,00 €.</t>
         </is>
@@ -1673,7 +1931,7 @@
       <c r="A17" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Sito web dello studio, Google Maps (foto, recensioni) e scheda Pagine Gialle.</t>
         </is>

</xml_diff>